<commit_message>
Løst problemet med at jeg ikke kunne hente Nikkei og China med "PS" eller PO samt lavet returns dataframe
</commit_message>
<xml_diff>
--- a/Future oversigt.xlsx
+++ b/Future oversigt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nykredit-my.sharepoint.com/personal/case_nykredit_dk/Documents/Dokumenter/Python projekter/Risk-Parity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{27D91E94-ADEF-4316-B385-AD4A97693817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF6DCD00-FBA9-4C24-BE10-225DC72B9D24}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{27D91E94-ADEF-4316-B385-AD4A97693817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{527DBBB6-C27C-4336-9094-D6BFA3D7F350}"/>
   <bookViews>
-    <workbookView xWindow="41235" yWindow="3555" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{374CA234-C103-4D78-B900-072EFD949F2A}"/>
+    <workbookView xWindow="41235" yWindow="3555" windowWidth="28800" windowHeight="15345" xr2:uid="{374CA234-C103-4D78-B900-072EFD949F2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <author>Casper Egon Hansen</author>
   </authors>
   <commentList>
-    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{0D97B504-CF4E-4C4E-9C03-6C76D76F27AC}">
+    <comment ref="C6" authorId="0" shapeId="0" xr:uid="{668AB6B0-C444-4BC1-BC91-20605C640CF7}">
       <text>
         <r>
           <rPr>
@@ -275,7 +275,7 @@
       <tp t="s">
         <v>Name</v>
         <stp/>
-        <stp>2</stp>
+        <stp>4</stp>
         <stp>101635421</stp>
         <tr r="C6" s="2"/>
       </tp>
@@ -2205,7 +2205,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CF7959D-DBD7-4DB0-B664-91C827A791A1}">
-  <dimension ref="C6:E3921"/>
+  <dimension ref="C6:E5226"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.125" bestFit="1" customWidth="1"/>
@@ -45290,6 +45290,3921 @@
         <v>14716</v>
       </c>
     </row>
+    <row r="3922" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3922" s="4"/>
+    </row>
+    <row r="3923" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3923" s="4"/>
+    </row>
+    <row r="3924" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3924" s="4"/>
+    </row>
+    <row r="3925" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3925" s="4"/>
+    </row>
+    <row r="3926" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3926" s="4"/>
+    </row>
+    <row r="3927" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3927" s="4"/>
+    </row>
+    <row r="3928" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3928" s="4"/>
+    </row>
+    <row r="3929" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3929" s="4"/>
+    </row>
+    <row r="3930" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3930" s="4"/>
+    </row>
+    <row r="3931" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3931" s="4"/>
+    </row>
+    <row r="3932" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3932" s="4"/>
+    </row>
+    <row r="3933" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3933" s="4"/>
+    </row>
+    <row r="3934" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3934" s="4"/>
+    </row>
+    <row r="3935" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3935" s="4"/>
+    </row>
+    <row r="3936" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C3936" s="4"/>
+    </row>
+    <row r="3937" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3937" s="4"/>
+    </row>
+    <row r="3938" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3938" s="4"/>
+    </row>
+    <row r="3939" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3939" s="4"/>
+    </row>
+    <row r="3940" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3940" s="4"/>
+    </row>
+    <row r="3941" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3941" s="4"/>
+    </row>
+    <row r="3942" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3942" s="4"/>
+    </row>
+    <row r="3943" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3943" s="4"/>
+    </row>
+    <row r="3944" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3944" s="4"/>
+    </row>
+    <row r="3945" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3945" s="4"/>
+    </row>
+    <row r="3946" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3946" s="4"/>
+    </row>
+    <row r="3947" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3947" s="4"/>
+    </row>
+    <row r="3948" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3948" s="4"/>
+    </row>
+    <row r="3949" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3949" s="4"/>
+    </row>
+    <row r="3950" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3950" s="4"/>
+    </row>
+    <row r="3951" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3951" s="4"/>
+    </row>
+    <row r="3952" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3952" s="4"/>
+    </row>
+    <row r="3953" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3953" s="4"/>
+    </row>
+    <row r="3954" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3954" s="4"/>
+    </row>
+    <row r="3955" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3955" s="4"/>
+    </row>
+    <row r="3956" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3956" s="4"/>
+    </row>
+    <row r="3957" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3957" s="4"/>
+    </row>
+    <row r="3958" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3958" s="4"/>
+    </row>
+    <row r="3959" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3959" s="4"/>
+    </row>
+    <row r="3960" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3960" s="4"/>
+    </row>
+    <row r="3961" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3961" s="4"/>
+    </row>
+    <row r="3962" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3962" s="4"/>
+    </row>
+    <row r="3963" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3963" s="4"/>
+    </row>
+    <row r="3964" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3964" s="4"/>
+    </row>
+    <row r="3965" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3965" s="4"/>
+    </row>
+    <row r="3966" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3966" s="4"/>
+    </row>
+    <row r="3967" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3967" s="4"/>
+    </row>
+    <row r="3968" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3968" s="4"/>
+    </row>
+    <row r="3969" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3969" s="4"/>
+    </row>
+    <row r="3970" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3970" s="4"/>
+    </row>
+    <row r="3971" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3971" s="4"/>
+    </row>
+    <row r="3972" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3972" s="4"/>
+    </row>
+    <row r="3973" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3973" s="4"/>
+    </row>
+    <row r="3974" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3974" s="4"/>
+    </row>
+    <row r="3975" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3975" s="4"/>
+    </row>
+    <row r="3976" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3976" s="4"/>
+    </row>
+    <row r="3977" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3977" s="4"/>
+    </row>
+    <row r="3978" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3978" s="4"/>
+    </row>
+    <row r="3979" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3979" s="4"/>
+    </row>
+    <row r="3980" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3980" s="4"/>
+    </row>
+    <row r="3981" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3981" s="4"/>
+    </row>
+    <row r="3982" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3982" s="4"/>
+    </row>
+    <row r="3983" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3983" s="4"/>
+    </row>
+    <row r="3984" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3984" s="4"/>
+    </row>
+    <row r="3985" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3985" s="4"/>
+    </row>
+    <row r="3986" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3986" s="4"/>
+    </row>
+    <row r="3987" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3987" s="4"/>
+    </row>
+    <row r="3988" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3988" s="4"/>
+    </row>
+    <row r="3989" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3989" s="4"/>
+    </row>
+    <row r="3990" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3990" s="4"/>
+    </row>
+    <row r="3991" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3991" s="4"/>
+    </row>
+    <row r="3992" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3992" s="4"/>
+    </row>
+    <row r="3993" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3993" s="4"/>
+    </row>
+    <row r="3994" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3994" s="4"/>
+    </row>
+    <row r="3995" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3995" s="4"/>
+    </row>
+    <row r="3996" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3996" s="4"/>
+    </row>
+    <row r="3997" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3997" s="4"/>
+    </row>
+    <row r="3998" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3998" s="4"/>
+    </row>
+    <row r="3999" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C3999" s="4"/>
+    </row>
+    <row r="4000" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4000" s="4"/>
+    </row>
+    <row r="4001" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4001" s="4"/>
+    </row>
+    <row r="4002" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4002" s="4"/>
+    </row>
+    <row r="4003" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4003" s="4"/>
+    </row>
+    <row r="4004" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4004" s="4"/>
+    </row>
+    <row r="4005" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4005" s="4"/>
+    </row>
+    <row r="4006" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4006" s="4"/>
+    </row>
+    <row r="4007" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4007" s="4"/>
+    </row>
+    <row r="4008" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4008" s="4"/>
+    </row>
+    <row r="4009" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4009" s="4"/>
+    </row>
+    <row r="4010" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4010" s="4"/>
+    </row>
+    <row r="4011" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4011" s="4"/>
+    </row>
+    <row r="4012" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4012" s="4"/>
+    </row>
+    <row r="4013" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4013" s="4"/>
+    </row>
+    <row r="4014" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4014" s="4"/>
+    </row>
+    <row r="4015" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4015" s="4"/>
+    </row>
+    <row r="4016" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4016" s="4"/>
+    </row>
+    <row r="4017" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4017" s="4"/>
+    </row>
+    <row r="4018" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4018" s="4"/>
+    </row>
+    <row r="4019" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4019" s="4"/>
+    </row>
+    <row r="4020" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4020" s="4"/>
+    </row>
+    <row r="4021" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4021" s="4"/>
+    </row>
+    <row r="4022" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4022" s="4"/>
+    </row>
+    <row r="4023" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4023" s="4"/>
+    </row>
+    <row r="4024" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4024" s="4"/>
+    </row>
+    <row r="4025" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4025" s="4"/>
+    </row>
+    <row r="4026" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4026" s="4"/>
+    </row>
+    <row r="4027" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4027" s="4"/>
+    </row>
+    <row r="4028" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4028" s="4"/>
+    </row>
+    <row r="4029" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4029" s="4"/>
+    </row>
+    <row r="4030" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4030" s="4"/>
+    </row>
+    <row r="4031" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4031" s="4"/>
+    </row>
+    <row r="4032" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4032" s="4"/>
+    </row>
+    <row r="4033" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4033" s="4"/>
+    </row>
+    <row r="4034" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4034" s="4"/>
+    </row>
+    <row r="4035" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4035" s="4"/>
+    </row>
+    <row r="4036" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4036" s="4"/>
+    </row>
+    <row r="4037" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4037" s="4"/>
+    </row>
+    <row r="4038" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4038" s="4"/>
+    </row>
+    <row r="4039" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4039" s="4"/>
+    </row>
+    <row r="4040" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4040" s="4"/>
+    </row>
+    <row r="4041" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4041" s="4"/>
+    </row>
+    <row r="4042" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4042" s="4"/>
+    </row>
+    <row r="4043" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4043" s="4"/>
+    </row>
+    <row r="4044" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4044" s="4"/>
+    </row>
+    <row r="4045" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4045" s="4"/>
+    </row>
+    <row r="4046" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4046" s="4"/>
+    </row>
+    <row r="4047" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4047" s="4"/>
+    </row>
+    <row r="4048" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4048" s="4"/>
+    </row>
+    <row r="4049" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4049" s="4"/>
+    </row>
+    <row r="4050" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4050" s="4"/>
+    </row>
+    <row r="4051" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4051" s="4"/>
+    </row>
+    <row r="4052" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4052" s="4"/>
+    </row>
+    <row r="4053" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4053" s="4"/>
+    </row>
+    <row r="4054" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4054" s="4"/>
+    </row>
+    <row r="4055" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4055" s="4"/>
+    </row>
+    <row r="4056" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4056" s="4"/>
+    </row>
+    <row r="4057" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4057" s="4"/>
+    </row>
+    <row r="4058" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4058" s="4"/>
+    </row>
+    <row r="4059" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4059" s="4"/>
+    </row>
+    <row r="4060" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4060" s="4"/>
+    </row>
+    <row r="4061" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4061" s="4"/>
+    </row>
+    <row r="4062" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4062" s="4"/>
+    </row>
+    <row r="4063" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4063" s="4"/>
+    </row>
+    <row r="4064" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4064" s="4"/>
+    </row>
+    <row r="4065" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4065" s="4"/>
+    </row>
+    <row r="4066" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4066" s="4"/>
+    </row>
+    <row r="4067" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4067" s="4"/>
+    </row>
+    <row r="4068" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4068" s="4"/>
+    </row>
+    <row r="4069" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4069" s="4"/>
+    </row>
+    <row r="4070" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4070" s="4"/>
+    </row>
+    <row r="4071" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4071" s="4"/>
+    </row>
+    <row r="4072" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4072" s="4"/>
+    </row>
+    <row r="4073" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4073" s="4"/>
+    </row>
+    <row r="4074" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4074" s="4"/>
+    </row>
+    <row r="4075" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4075" s="4"/>
+    </row>
+    <row r="4076" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4076" s="4"/>
+    </row>
+    <row r="4077" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4077" s="4"/>
+    </row>
+    <row r="4078" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4078" s="4"/>
+    </row>
+    <row r="4079" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4079" s="4"/>
+    </row>
+    <row r="4080" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4080" s="4"/>
+    </row>
+    <row r="4081" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4081" s="4"/>
+    </row>
+    <row r="4082" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4082" s="4"/>
+    </row>
+    <row r="4083" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4083" s="4"/>
+    </row>
+    <row r="4084" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4084" s="4"/>
+    </row>
+    <row r="4085" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4085" s="4"/>
+    </row>
+    <row r="4086" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4086" s="4"/>
+    </row>
+    <row r="4087" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4087" s="4"/>
+    </row>
+    <row r="4088" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4088" s="4"/>
+    </row>
+    <row r="4089" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4089" s="4"/>
+    </row>
+    <row r="4090" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4090" s="4"/>
+    </row>
+    <row r="4091" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4091" s="4"/>
+    </row>
+    <row r="4092" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4092" s="4"/>
+    </row>
+    <row r="4093" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4093" s="4"/>
+    </row>
+    <row r="4094" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4094" s="4"/>
+    </row>
+    <row r="4095" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4095" s="4"/>
+    </row>
+    <row r="4096" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4096" s="4"/>
+    </row>
+    <row r="4097" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4097" s="4"/>
+    </row>
+    <row r="4098" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4098" s="4"/>
+    </row>
+    <row r="4099" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4099" s="4"/>
+    </row>
+    <row r="4100" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4100" s="4"/>
+    </row>
+    <row r="4101" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4101" s="4"/>
+    </row>
+    <row r="4102" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4102" s="4"/>
+    </row>
+    <row r="4103" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4103" s="4"/>
+    </row>
+    <row r="4104" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4104" s="4"/>
+    </row>
+    <row r="4105" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4105" s="4"/>
+    </row>
+    <row r="4106" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4106" s="4"/>
+    </row>
+    <row r="4107" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4107" s="4"/>
+    </row>
+    <row r="4108" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4108" s="4"/>
+    </row>
+    <row r="4109" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4109" s="4"/>
+    </row>
+    <row r="4110" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4110" s="4"/>
+    </row>
+    <row r="4111" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4111" s="4"/>
+    </row>
+    <row r="4112" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4112" s="4"/>
+    </row>
+    <row r="4113" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4113" s="4"/>
+    </row>
+    <row r="4114" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4114" s="4"/>
+    </row>
+    <row r="4115" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4115" s="4"/>
+    </row>
+    <row r="4116" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4116" s="4"/>
+    </row>
+    <row r="4117" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4117" s="4"/>
+    </row>
+    <row r="4118" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4118" s="4"/>
+    </row>
+    <row r="4119" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4119" s="4"/>
+    </row>
+    <row r="4120" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4120" s="4"/>
+    </row>
+    <row r="4121" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4121" s="4"/>
+    </row>
+    <row r="4122" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4122" s="4"/>
+    </row>
+    <row r="4123" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4123" s="4"/>
+    </row>
+    <row r="4124" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4124" s="4"/>
+    </row>
+    <row r="4125" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4125" s="4"/>
+    </row>
+    <row r="4126" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4126" s="4"/>
+    </row>
+    <row r="4127" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4127" s="4"/>
+    </row>
+    <row r="4128" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4128" s="4"/>
+    </row>
+    <row r="4129" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4129" s="4"/>
+    </row>
+    <row r="4130" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4130" s="4"/>
+    </row>
+    <row r="4131" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4131" s="4"/>
+    </row>
+    <row r="4132" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4132" s="4"/>
+    </row>
+    <row r="4133" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4133" s="4"/>
+    </row>
+    <row r="4134" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4134" s="4"/>
+    </row>
+    <row r="4135" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4135" s="4"/>
+    </row>
+    <row r="4136" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4136" s="4"/>
+    </row>
+    <row r="4137" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4137" s="4"/>
+    </row>
+    <row r="4138" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4138" s="4"/>
+    </row>
+    <row r="4139" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4139" s="4"/>
+    </row>
+    <row r="4140" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4140" s="4"/>
+    </row>
+    <row r="4141" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4141" s="4"/>
+    </row>
+    <row r="4142" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4142" s="4"/>
+    </row>
+    <row r="4143" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4143" s="4"/>
+    </row>
+    <row r="4144" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4144" s="4"/>
+    </row>
+    <row r="4145" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4145" s="4"/>
+    </row>
+    <row r="4146" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4146" s="4"/>
+    </row>
+    <row r="4147" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4147" s="4"/>
+    </row>
+    <row r="4148" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4148" s="4"/>
+    </row>
+    <row r="4149" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4149" s="4"/>
+    </row>
+    <row r="4150" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4150" s="4"/>
+    </row>
+    <row r="4151" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4151" s="4"/>
+    </row>
+    <row r="4152" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4152" s="4"/>
+    </row>
+    <row r="4153" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4153" s="4"/>
+    </row>
+    <row r="4154" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4154" s="4"/>
+    </row>
+    <row r="4155" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4155" s="4"/>
+    </row>
+    <row r="4156" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4156" s="4"/>
+    </row>
+    <row r="4157" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4157" s="4"/>
+    </row>
+    <row r="4158" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4158" s="4"/>
+    </row>
+    <row r="4159" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4159" s="4"/>
+    </row>
+    <row r="4160" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4160" s="4"/>
+    </row>
+    <row r="4161" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4161" s="4"/>
+    </row>
+    <row r="4162" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4162" s="4"/>
+    </row>
+    <row r="4163" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4163" s="4"/>
+    </row>
+    <row r="4164" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4164" s="4"/>
+    </row>
+    <row r="4165" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4165" s="4"/>
+    </row>
+    <row r="4166" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4166" s="4"/>
+    </row>
+    <row r="4167" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4167" s="4"/>
+    </row>
+    <row r="4168" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4168" s="4"/>
+    </row>
+    <row r="4169" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4169" s="4"/>
+    </row>
+    <row r="4170" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4170" s="4"/>
+    </row>
+    <row r="4171" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4171" s="4"/>
+    </row>
+    <row r="4172" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4172" s="4"/>
+    </row>
+    <row r="4173" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4173" s="4"/>
+    </row>
+    <row r="4174" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4174" s="4"/>
+    </row>
+    <row r="4175" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4175" s="4"/>
+    </row>
+    <row r="4176" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4176" s="4"/>
+    </row>
+    <row r="4177" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4177" s="4"/>
+    </row>
+    <row r="4178" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4178" s="4"/>
+    </row>
+    <row r="4179" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4179" s="4"/>
+    </row>
+    <row r="4180" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4180" s="4"/>
+    </row>
+    <row r="4181" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4181" s="4"/>
+    </row>
+    <row r="4182" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4182" s="4"/>
+    </row>
+    <row r="4183" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4183" s="4"/>
+    </row>
+    <row r="4184" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4184" s="4"/>
+    </row>
+    <row r="4185" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4185" s="4"/>
+    </row>
+    <row r="4186" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4186" s="4"/>
+    </row>
+    <row r="4187" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4187" s="4"/>
+    </row>
+    <row r="4188" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4188" s="4"/>
+    </row>
+    <row r="4189" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4189" s="4"/>
+    </row>
+    <row r="4190" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4190" s="4"/>
+    </row>
+    <row r="4191" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4191" s="4"/>
+    </row>
+    <row r="4192" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4192" s="4"/>
+    </row>
+    <row r="4193" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4193" s="4"/>
+    </row>
+    <row r="4194" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4194" s="4"/>
+    </row>
+    <row r="4195" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4195" s="4"/>
+    </row>
+    <row r="4196" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4196" s="4"/>
+    </row>
+    <row r="4197" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4197" s="4"/>
+    </row>
+    <row r="4198" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4198" s="4"/>
+    </row>
+    <row r="4199" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4199" s="4"/>
+    </row>
+    <row r="4200" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4200" s="4"/>
+    </row>
+    <row r="4201" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4201" s="4"/>
+    </row>
+    <row r="4202" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4202" s="4"/>
+    </row>
+    <row r="4203" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4203" s="4"/>
+    </row>
+    <row r="4204" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4204" s="4"/>
+    </row>
+    <row r="4205" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4205" s="4"/>
+    </row>
+    <row r="4206" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4206" s="4"/>
+    </row>
+    <row r="4207" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4207" s="4"/>
+    </row>
+    <row r="4208" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4208" s="4"/>
+    </row>
+    <row r="4209" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4209" s="4"/>
+    </row>
+    <row r="4210" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4210" s="4"/>
+    </row>
+    <row r="4211" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4211" s="4"/>
+    </row>
+    <row r="4212" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4212" s="4"/>
+    </row>
+    <row r="4213" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4213" s="4"/>
+    </row>
+    <row r="4214" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4214" s="4"/>
+    </row>
+    <row r="4215" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4215" s="4"/>
+    </row>
+    <row r="4216" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4216" s="4"/>
+    </row>
+    <row r="4217" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4217" s="4"/>
+    </row>
+    <row r="4218" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4218" s="4"/>
+    </row>
+    <row r="4219" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4219" s="4"/>
+    </row>
+    <row r="4220" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4220" s="4"/>
+    </row>
+    <row r="4221" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4221" s="4"/>
+    </row>
+    <row r="4222" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4222" s="4"/>
+    </row>
+    <row r="4223" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4223" s="4"/>
+    </row>
+    <row r="4224" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4224" s="4"/>
+    </row>
+    <row r="4225" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4225" s="4"/>
+    </row>
+    <row r="4226" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4226" s="4"/>
+    </row>
+    <row r="4227" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4227" s="4"/>
+    </row>
+    <row r="4228" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4228" s="4"/>
+    </row>
+    <row r="4229" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4229" s="4"/>
+    </row>
+    <row r="4230" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4230" s="4"/>
+    </row>
+    <row r="4231" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4231" s="4"/>
+    </row>
+    <row r="4232" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4232" s="4"/>
+    </row>
+    <row r="4233" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4233" s="4"/>
+    </row>
+    <row r="4234" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4234" s="4"/>
+    </row>
+    <row r="4235" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4235" s="4"/>
+    </row>
+    <row r="4236" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4236" s="4"/>
+    </row>
+    <row r="4237" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4237" s="4"/>
+    </row>
+    <row r="4238" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4238" s="4"/>
+    </row>
+    <row r="4239" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4239" s="4"/>
+    </row>
+    <row r="4240" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4240" s="4"/>
+    </row>
+    <row r="4241" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4241" s="4"/>
+    </row>
+    <row r="4242" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4242" s="4"/>
+    </row>
+    <row r="4243" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4243" s="4"/>
+    </row>
+    <row r="4244" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4244" s="4"/>
+    </row>
+    <row r="4245" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4245" s="4"/>
+    </row>
+    <row r="4246" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4246" s="4"/>
+    </row>
+    <row r="4247" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4247" s="4"/>
+    </row>
+    <row r="4248" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4248" s="4"/>
+    </row>
+    <row r="4249" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4249" s="4"/>
+    </row>
+    <row r="4250" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4250" s="4"/>
+    </row>
+    <row r="4251" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4251" s="4"/>
+    </row>
+    <row r="4252" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4252" s="4"/>
+    </row>
+    <row r="4253" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4253" s="4"/>
+    </row>
+    <row r="4254" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4254" s="4"/>
+    </row>
+    <row r="4255" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4255" s="4"/>
+    </row>
+    <row r="4256" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4256" s="4"/>
+    </row>
+    <row r="4257" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4257" s="4"/>
+    </row>
+    <row r="4258" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4258" s="4"/>
+    </row>
+    <row r="4259" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4259" s="4"/>
+    </row>
+    <row r="4260" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4260" s="4"/>
+    </row>
+    <row r="4261" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4261" s="4"/>
+    </row>
+    <row r="4262" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4262" s="4"/>
+    </row>
+    <row r="4263" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4263" s="4"/>
+    </row>
+    <row r="4264" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4264" s="4"/>
+    </row>
+    <row r="4265" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4265" s="4"/>
+    </row>
+    <row r="4266" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4266" s="4"/>
+    </row>
+    <row r="4267" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4267" s="4"/>
+    </row>
+    <row r="4268" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4268" s="4"/>
+    </row>
+    <row r="4269" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4269" s="4"/>
+    </row>
+    <row r="4270" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4270" s="4"/>
+    </row>
+    <row r="4271" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4271" s="4"/>
+    </row>
+    <row r="4272" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4272" s="4"/>
+    </row>
+    <row r="4273" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4273" s="4"/>
+    </row>
+    <row r="4274" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4274" s="4"/>
+    </row>
+    <row r="4275" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4275" s="4"/>
+    </row>
+    <row r="4276" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4276" s="4"/>
+    </row>
+    <row r="4277" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4277" s="4"/>
+    </row>
+    <row r="4278" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4278" s="4"/>
+    </row>
+    <row r="4279" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4279" s="4"/>
+    </row>
+    <row r="4280" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4280" s="4"/>
+    </row>
+    <row r="4281" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4281" s="4"/>
+    </row>
+    <row r="4282" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4282" s="4"/>
+    </row>
+    <row r="4283" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4283" s="4"/>
+    </row>
+    <row r="4284" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4284" s="4"/>
+    </row>
+    <row r="4285" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4285" s="4"/>
+    </row>
+    <row r="4286" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4286" s="4"/>
+    </row>
+    <row r="4287" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4287" s="4"/>
+    </row>
+    <row r="4288" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4288" s="4"/>
+    </row>
+    <row r="4289" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4289" s="4"/>
+    </row>
+    <row r="4290" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4290" s="4"/>
+    </row>
+    <row r="4291" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4291" s="4"/>
+    </row>
+    <row r="4292" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4292" s="4"/>
+    </row>
+    <row r="4293" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4293" s="4"/>
+    </row>
+    <row r="4294" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4294" s="4"/>
+    </row>
+    <row r="4295" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4295" s="4"/>
+    </row>
+    <row r="4296" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4296" s="4"/>
+    </row>
+    <row r="4297" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4297" s="4"/>
+    </row>
+    <row r="4298" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4298" s="4"/>
+    </row>
+    <row r="4299" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4299" s="4"/>
+    </row>
+    <row r="4300" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4300" s="4"/>
+    </row>
+    <row r="4301" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4301" s="4"/>
+    </row>
+    <row r="4302" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4302" s="4"/>
+    </row>
+    <row r="4303" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4303" s="4"/>
+    </row>
+    <row r="4304" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4304" s="4"/>
+    </row>
+    <row r="4305" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4305" s="4"/>
+    </row>
+    <row r="4306" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4306" s="4"/>
+    </row>
+    <row r="4307" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4307" s="4"/>
+    </row>
+    <row r="4308" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4308" s="4"/>
+    </row>
+    <row r="4309" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4309" s="4"/>
+    </row>
+    <row r="4310" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4310" s="4"/>
+    </row>
+    <row r="4311" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4311" s="4"/>
+    </row>
+    <row r="4312" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4312" s="4"/>
+    </row>
+    <row r="4313" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4313" s="4"/>
+    </row>
+    <row r="4314" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4314" s="4"/>
+    </row>
+    <row r="4315" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4315" s="4"/>
+    </row>
+    <row r="4316" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4316" s="4"/>
+    </row>
+    <row r="4317" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4317" s="4"/>
+    </row>
+    <row r="4318" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4318" s="4"/>
+    </row>
+    <row r="4319" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4319" s="4"/>
+    </row>
+    <row r="4320" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4320" s="4"/>
+    </row>
+    <row r="4321" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4321" s="4"/>
+    </row>
+    <row r="4322" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4322" s="4"/>
+    </row>
+    <row r="4323" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4323" s="4"/>
+    </row>
+    <row r="4324" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4324" s="4"/>
+    </row>
+    <row r="4325" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4325" s="4"/>
+    </row>
+    <row r="4326" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4326" s="4"/>
+    </row>
+    <row r="4327" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4327" s="4"/>
+    </row>
+    <row r="4328" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4328" s="4"/>
+    </row>
+    <row r="4329" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4329" s="4"/>
+    </row>
+    <row r="4330" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4330" s="4"/>
+    </row>
+    <row r="4331" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4331" s="4"/>
+    </row>
+    <row r="4332" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4332" s="4"/>
+    </row>
+    <row r="4333" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4333" s="4"/>
+    </row>
+    <row r="4334" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4334" s="4"/>
+    </row>
+    <row r="4335" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4335" s="4"/>
+    </row>
+    <row r="4336" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4336" s="4"/>
+    </row>
+    <row r="4337" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4337" s="4"/>
+    </row>
+    <row r="4338" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4338" s="4"/>
+    </row>
+    <row r="4339" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4339" s="4"/>
+    </row>
+    <row r="4340" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4340" s="4"/>
+    </row>
+    <row r="4341" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4341" s="4"/>
+    </row>
+    <row r="4342" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4342" s="4"/>
+    </row>
+    <row r="4343" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4343" s="4"/>
+    </row>
+    <row r="4344" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4344" s="4"/>
+    </row>
+    <row r="4345" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4345" s="4"/>
+    </row>
+    <row r="4346" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4346" s="4"/>
+    </row>
+    <row r="4347" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4347" s="4"/>
+    </row>
+    <row r="4348" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4348" s="4"/>
+    </row>
+    <row r="4349" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4349" s="4"/>
+    </row>
+    <row r="4350" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4350" s="4"/>
+    </row>
+    <row r="4351" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4351" s="4"/>
+    </row>
+    <row r="4352" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4352" s="4"/>
+    </row>
+    <row r="4353" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4353" s="4"/>
+    </row>
+    <row r="4354" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4354" s="4"/>
+    </row>
+    <row r="4355" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4355" s="4"/>
+    </row>
+    <row r="4356" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4356" s="4"/>
+    </row>
+    <row r="4357" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4357" s="4"/>
+    </row>
+    <row r="4358" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4358" s="4"/>
+    </row>
+    <row r="4359" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4359" s="4"/>
+    </row>
+    <row r="4360" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4360" s="4"/>
+    </row>
+    <row r="4361" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4361" s="4"/>
+    </row>
+    <row r="4362" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4362" s="4"/>
+    </row>
+    <row r="4363" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4363" s="4"/>
+    </row>
+    <row r="4364" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4364" s="4"/>
+    </row>
+    <row r="4365" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4365" s="4"/>
+    </row>
+    <row r="4366" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4366" s="4"/>
+    </row>
+    <row r="4367" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4367" s="4"/>
+    </row>
+    <row r="4368" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4368" s="4"/>
+    </row>
+    <row r="4369" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4369" s="4"/>
+    </row>
+    <row r="4370" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4370" s="4"/>
+    </row>
+    <row r="4371" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4371" s="4"/>
+    </row>
+    <row r="4372" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4372" s="4"/>
+    </row>
+    <row r="4373" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4373" s="4"/>
+    </row>
+    <row r="4374" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4374" s="4"/>
+    </row>
+    <row r="4375" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4375" s="4"/>
+    </row>
+    <row r="4376" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4376" s="4"/>
+    </row>
+    <row r="4377" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4377" s="4"/>
+    </row>
+    <row r="4378" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4378" s="4"/>
+    </row>
+    <row r="4379" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4379" s="4"/>
+    </row>
+    <row r="4380" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4380" s="4"/>
+    </row>
+    <row r="4381" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4381" s="4"/>
+    </row>
+    <row r="4382" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4382" s="4"/>
+    </row>
+    <row r="4383" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4383" s="4"/>
+    </row>
+    <row r="4384" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4384" s="4"/>
+    </row>
+    <row r="4385" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4385" s="4"/>
+    </row>
+    <row r="4386" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4386" s="4"/>
+    </row>
+    <row r="4387" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4387" s="4"/>
+    </row>
+    <row r="4388" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4388" s="4"/>
+    </row>
+    <row r="4389" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4389" s="4"/>
+    </row>
+    <row r="4390" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4390" s="4"/>
+    </row>
+    <row r="4391" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4391" s="4"/>
+    </row>
+    <row r="4392" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4392" s="4"/>
+    </row>
+    <row r="4393" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4393" s="4"/>
+    </row>
+    <row r="4394" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4394" s="4"/>
+    </row>
+    <row r="4395" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4395" s="4"/>
+    </row>
+    <row r="4396" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4396" s="4"/>
+    </row>
+    <row r="4397" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4397" s="4"/>
+    </row>
+    <row r="4398" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4398" s="4"/>
+    </row>
+    <row r="4399" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4399" s="4"/>
+    </row>
+    <row r="4400" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4400" s="4"/>
+    </row>
+    <row r="4401" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4401" s="4"/>
+    </row>
+    <row r="4402" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4402" s="4"/>
+    </row>
+    <row r="4403" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4403" s="4"/>
+    </row>
+    <row r="4404" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4404" s="4"/>
+    </row>
+    <row r="4405" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4405" s="4"/>
+    </row>
+    <row r="4406" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4406" s="4"/>
+    </row>
+    <row r="4407" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4407" s="4"/>
+    </row>
+    <row r="4408" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4408" s="4"/>
+    </row>
+    <row r="4409" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4409" s="4"/>
+    </row>
+    <row r="4410" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4410" s="4"/>
+    </row>
+    <row r="4411" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4411" s="4"/>
+    </row>
+    <row r="4412" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4412" s="4"/>
+    </row>
+    <row r="4413" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4413" s="4"/>
+    </row>
+    <row r="4414" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4414" s="4"/>
+    </row>
+    <row r="4415" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4415" s="4"/>
+    </row>
+    <row r="4416" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4416" s="4"/>
+    </row>
+    <row r="4417" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4417" s="4"/>
+    </row>
+    <row r="4418" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4418" s="4"/>
+    </row>
+    <row r="4419" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4419" s="4"/>
+    </row>
+    <row r="4420" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4420" s="4"/>
+    </row>
+    <row r="4421" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4421" s="4"/>
+    </row>
+    <row r="4422" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4422" s="4"/>
+    </row>
+    <row r="4423" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4423" s="4"/>
+    </row>
+    <row r="4424" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4424" s="4"/>
+    </row>
+    <row r="4425" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4425" s="4"/>
+    </row>
+    <row r="4426" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4426" s="4"/>
+    </row>
+    <row r="4427" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4427" s="4"/>
+    </row>
+    <row r="4428" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4428" s="4"/>
+    </row>
+    <row r="4429" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4429" s="4"/>
+    </row>
+    <row r="4430" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4430" s="4"/>
+    </row>
+    <row r="4431" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4431" s="4"/>
+    </row>
+    <row r="4432" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4432" s="4"/>
+    </row>
+    <row r="4433" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4433" s="4"/>
+    </row>
+    <row r="4434" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4434" s="4"/>
+    </row>
+    <row r="4435" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4435" s="4"/>
+    </row>
+    <row r="4436" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4436" s="4"/>
+    </row>
+    <row r="4437" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4437" s="4"/>
+    </row>
+    <row r="4438" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4438" s="4"/>
+    </row>
+    <row r="4439" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4439" s="4"/>
+    </row>
+    <row r="4440" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4440" s="4"/>
+    </row>
+    <row r="4441" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4441" s="4"/>
+    </row>
+    <row r="4442" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4442" s="4"/>
+    </row>
+    <row r="4443" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4443" s="4"/>
+    </row>
+    <row r="4444" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4444" s="4"/>
+    </row>
+    <row r="4445" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4445" s="4"/>
+    </row>
+    <row r="4446" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4446" s="4"/>
+    </row>
+    <row r="4447" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4447" s="4"/>
+    </row>
+    <row r="4448" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4448" s="4"/>
+    </row>
+    <row r="4449" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4449" s="4"/>
+    </row>
+    <row r="4450" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4450" s="4"/>
+    </row>
+    <row r="4451" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4451" s="4"/>
+    </row>
+    <row r="4452" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4452" s="4"/>
+    </row>
+    <row r="4453" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4453" s="4"/>
+    </row>
+    <row r="4454" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4454" s="4"/>
+    </row>
+    <row r="4455" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4455" s="4"/>
+    </row>
+    <row r="4456" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4456" s="4"/>
+    </row>
+    <row r="4457" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4457" s="4"/>
+    </row>
+    <row r="4458" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4458" s="4"/>
+    </row>
+    <row r="4459" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4459" s="4"/>
+    </row>
+    <row r="4460" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4460" s="4"/>
+    </row>
+    <row r="4461" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4461" s="4"/>
+    </row>
+    <row r="4462" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4462" s="4"/>
+    </row>
+    <row r="4463" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4463" s="4"/>
+    </row>
+    <row r="4464" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4464" s="4"/>
+    </row>
+    <row r="4465" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4465" s="4"/>
+    </row>
+    <row r="4466" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4466" s="4"/>
+    </row>
+    <row r="4467" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4467" s="4"/>
+    </row>
+    <row r="4468" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4468" s="4"/>
+    </row>
+    <row r="4469" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4469" s="4"/>
+    </row>
+    <row r="4470" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4470" s="4"/>
+    </row>
+    <row r="4471" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4471" s="4"/>
+    </row>
+    <row r="4472" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4472" s="4"/>
+    </row>
+    <row r="4473" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4473" s="4"/>
+    </row>
+    <row r="4474" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4474" s="4"/>
+    </row>
+    <row r="4475" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4475" s="4"/>
+    </row>
+    <row r="4476" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4476" s="4"/>
+    </row>
+    <row r="4477" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4477" s="4"/>
+    </row>
+    <row r="4478" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4478" s="4"/>
+    </row>
+    <row r="4479" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4479" s="4"/>
+    </row>
+    <row r="4480" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4480" s="4"/>
+    </row>
+    <row r="4481" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4481" s="4"/>
+    </row>
+    <row r="4482" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4482" s="4"/>
+    </row>
+    <row r="4483" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4483" s="4"/>
+    </row>
+    <row r="4484" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4484" s="4"/>
+    </row>
+    <row r="4485" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4485" s="4"/>
+    </row>
+    <row r="4486" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4486" s="4"/>
+    </row>
+    <row r="4487" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4487" s="4"/>
+    </row>
+    <row r="4488" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4488" s="4"/>
+    </row>
+    <row r="4489" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4489" s="4"/>
+    </row>
+    <row r="4490" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4490" s="4"/>
+    </row>
+    <row r="4491" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4491" s="4"/>
+    </row>
+    <row r="4492" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4492" s="4"/>
+    </row>
+    <row r="4493" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4493" s="4"/>
+    </row>
+    <row r="4494" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4494" s="4"/>
+    </row>
+    <row r="4495" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4495" s="4"/>
+    </row>
+    <row r="4496" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4496" s="4"/>
+    </row>
+    <row r="4497" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4497" s="4"/>
+    </row>
+    <row r="4498" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4498" s="4"/>
+    </row>
+    <row r="4499" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4499" s="4"/>
+    </row>
+    <row r="4500" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4500" s="4"/>
+    </row>
+    <row r="4501" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4501" s="4"/>
+    </row>
+    <row r="4502" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4502" s="4"/>
+    </row>
+    <row r="4503" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4503" s="4"/>
+    </row>
+    <row r="4504" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4504" s="4"/>
+    </row>
+    <row r="4505" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4505" s="4"/>
+    </row>
+    <row r="4506" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4506" s="4"/>
+    </row>
+    <row r="4507" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4507" s="4"/>
+    </row>
+    <row r="4508" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4508" s="4"/>
+    </row>
+    <row r="4509" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4509" s="4"/>
+    </row>
+    <row r="4510" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4510" s="4"/>
+    </row>
+    <row r="4511" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4511" s="4"/>
+    </row>
+    <row r="4512" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4512" s="4"/>
+    </row>
+    <row r="4513" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4513" s="4"/>
+    </row>
+    <row r="4514" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4514" s="4"/>
+    </row>
+    <row r="4515" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4515" s="4"/>
+    </row>
+    <row r="4516" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4516" s="4"/>
+    </row>
+    <row r="4517" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4517" s="4"/>
+    </row>
+    <row r="4518" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4518" s="4"/>
+    </row>
+    <row r="4519" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4519" s="4"/>
+    </row>
+    <row r="4520" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4520" s="4"/>
+    </row>
+    <row r="4521" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4521" s="4"/>
+    </row>
+    <row r="4522" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4522" s="4"/>
+    </row>
+    <row r="4523" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4523" s="4"/>
+    </row>
+    <row r="4524" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4524" s="4"/>
+    </row>
+    <row r="4525" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4525" s="4"/>
+    </row>
+    <row r="4526" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4526" s="4"/>
+    </row>
+    <row r="4527" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4527" s="4"/>
+    </row>
+    <row r="4528" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4528" s="4"/>
+    </row>
+    <row r="4529" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4529" s="4"/>
+    </row>
+    <row r="4530" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4530" s="4"/>
+    </row>
+    <row r="4531" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4531" s="4"/>
+    </row>
+    <row r="4532" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4532" s="4"/>
+    </row>
+    <row r="4533" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4533" s="4"/>
+    </row>
+    <row r="4534" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4534" s="4"/>
+    </row>
+    <row r="4535" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4535" s="4"/>
+    </row>
+    <row r="4536" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4536" s="4"/>
+    </row>
+    <row r="4537" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4537" s="4"/>
+    </row>
+    <row r="4538" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4538" s="4"/>
+    </row>
+    <row r="4539" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4539" s="4"/>
+    </row>
+    <row r="4540" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4540" s="4"/>
+    </row>
+    <row r="4541" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4541" s="4"/>
+    </row>
+    <row r="4542" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4542" s="4"/>
+    </row>
+    <row r="4543" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4543" s="4"/>
+    </row>
+    <row r="4544" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4544" s="4"/>
+    </row>
+    <row r="4545" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4545" s="4"/>
+    </row>
+    <row r="4546" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4546" s="4"/>
+    </row>
+    <row r="4547" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4547" s="4"/>
+    </row>
+    <row r="4548" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4548" s="4"/>
+    </row>
+    <row r="4549" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4549" s="4"/>
+    </row>
+    <row r="4550" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4550" s="4"/>
+    </row>
+    <row r="4551" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4551" s="4"/>
+    </row>
+    <row r="4552" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4552" s="4"/>
+    </row>
+    <row r="4553" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4553" s="4"/>
+    </row>
+    <row r="4554" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4554" s="4"/>
+    </row>
+    <row r="4555" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4555" s="4"/>
+    </row>
+    <row r="4556" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4556" s="4"/>
+    </row>
+    <row r="4557" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4557" s="4"/>
+    </row>
+    <row r="4558" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4558" s="4"/>
+    </row>
+    <row r="4559" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4559" s="4"/>
+    </row>
+    <row r="4560" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4560" s="4"/>
+    </row>
+    <row r="4561" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4561" s="4"/>
+    </row>
+    <row r="4562" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4562" s="4"/>
+    </row>
+    <row r="4563" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4563" s="4"/>
+    </row>
+    <row r="4564" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4564" s="4"/>
+    </row>
+    <row r="4565" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4565" s="4"/>
+    </row>
+    <row r="4566" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4566" s="4"/>
+    </row>
+    <row r="4567" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4567" s="4"/>
+    </row>
+    <row r="4568" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4568" s="4"/>
+    </row>
+    <row r="4569" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4569" s="4"/>
+    </row>
+    <row r="4570" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4570" s="4"/>
+    </row>
+    <row r="4571" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4571" s="4"/>
+    </row>
+    <row r="4572" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4572" s="4"/>
+    </row>
+    <row r="4573" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4573" s="4"/>
+    </row>
+    <row r="4574" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4574" s="4"/>
+    </row>
+    <row r="4575" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4575" s="4"/>
+    </row>
+    <row r="4576" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4576" s="4"/>
+    </row>
+    <row r="4577" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4577" s="4"/>
+    </row>
+    <row r="4578" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4578" s="4"/>
+    </row>
+    <row r="4579" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4579" s="4"/>
+    </row>
+    <row r="4580" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4580" s="4"/>
+    </row>
+    <row r="4581" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4581" s="4"/>
+    </row>
+    <row r="4582" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4582" s="4"/>
+    </row>
+    <row r="4583" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4583" s="4"/>
+    </row>
+    <row r="4584" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4584" s="4"/>
+    </row>
+    <row r="4585" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4585" s="4"/>
+    </row>
+    <row r="4586" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4586" s="4"/>
+    </row>
+    <row r="4587" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4587" s="4"/>
+    </row>
+    <row r="4588" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4588" s="4"/>
+    </row>
+    <row r="4589" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4589" s="4"/>
+    </row>
+    <row r="4590" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4590" s="4"/>
+    </row>
+    <row r="4591" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4591" s="4"/>
+    </row>
+    <row r="4592" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4592" s="4"/>
+    </row>
+    <row r="4593" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4593" s="4"/>
+    </row>
+    <row r="4594" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4594" s="4"/>
+    </row>
+    <row r="4595" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4595" s="4"/>
+    </row>
+    <row r="4596" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4596" s="4"/>
+    </row>
+    <row r="4597" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4597" s="4"/>
+    </row>
+    <row r="4598" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4598" s="4"/>
+    </row>
+    <row r="4599" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4599" s="4"/>
+    </row>
+    <row r="4600" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4600" s="4"/>
+    </row>
+    <row r="4601" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4601" s="4"/>
+    </row>
+    <row r="4602" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4602" s="4"/>
+    </row>
+    <row r="4603" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4603" s="4"/>
+    </row>
+    <row r="4604" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4604" s="4"/>
+    </row>
+    <row r="4605" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4605" s="4"/>
+    </row>
+    <row r="4606" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4606" s="4"/>
+    </row>
+    <row r="4607" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4607" s="4"/>
+    </row>
+    <row r="4608" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4608" s="4"/>
+    </row>
+    <row r="4609" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4609" s="4"/>
+    </row>
+    <row r="4610" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4610" s="4"/>
+    </row>
+    <row r="4611" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4611" s="4"/>
+    </row>
+    <row r="4612" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4612" s="4"/>
+    </row>
+    <row r="4613" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4613" s="4"/>
+    </row>
+    <row r="4614" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4614" s="4"/>
+    </row>
+    <row r="4615" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4615" s="4"/>
+    </row>
+    <row r="4616" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4616" s="4"/>
+    </row>
+    <row r="4617" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4617" s="4"/>
+    </row>
+    <row r="4618" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4618" s="4"/>
+    </row>
+    <row r="4619" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4619" s="4"/>
+    </row>
+    <row r="4620" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4620" s="4"/>
+    </row>
+    <row r="4621" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4621" s="4"/>
+    </row>
+    <row r="4622" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4622" s="4"/>
+    </row>
+    <row r="4623" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4623" s="4"/>
+    </row>
+    <row r="4624" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4624" s="4"/>
+    </row>
+    <row r="4625" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4625" s="4"/>
+    </row>
+    <row r="4626" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4626" s="4"/>
+    </row>
+    <row r="4627" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4627" s="4"/>
+    </row>
+    <row r="4628" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4628" s="4"/>
+    </row>
+    <row r="4629" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4629" s="4"/>
+    </row>
+    <row r="4630" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4630" s="4"/>
+    </row>
+    <row r="4631" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4631" s="4"/>
+    </row>
+    <row r="4632" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4632" s="4"/>
+    </row>
+    <row r="4633" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4633" s="4"/>
+    </row>
+    <row r="4634" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4634" s="4"/>
+    </row>
+    <row r="4635" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4635" s="4"/>
+    </row>
+    <row r="4636" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4636" s="4"/>
+    </row>
+    <row r="4637" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4637" s="4"/>
+    </row>
+    <row r="4638" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4638" s="4"/>
+    </row>
+    <row r="4639" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4639" s="4"/>
+    </row>
+    <row r="4640" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4640" s="4"/>
+    </row>
+    <row r="4641" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4641" s="4"/>
+    </row>
+    <row r="4642" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4642" s="4"/>
+    </row>
+    <row r="4643" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4643" s="4"/>
+    </row>
+    <row r="4644" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4644" s="4"/>
+    </row>
+    <row r="4645" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4645" s="4"/>
+    </row>
+    <row r="4646" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4646" s="4"/>
+    </row>
+    <row r="4647" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4647" s="4"/>
+    </row>
+    <row r="4648" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4648" s="4"/>
+    </row>
+    <row r="4649" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4649" s="4"/>
+    </row>
+    <row r="4650" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4650" s="4"/>
+    </row>
+    <row r="4651" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4651" s="4"/>
+    </row>
+    <row r="4652" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4652" s="4"/>
+    </row>
+    <row r="4653" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4653" s="4"/>
+    </row>
+    <row r="4654" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4654" s="4"/>
+    </row>
+    <row r="4655" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4655" s="4"/>
+    </row>
+    <row r="4656" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4656" s="4"/>
+    </row>
+    <row r="4657" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4657" s="4"/>
+    </row>
+    <row r="4658" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4658" s="4"/>
+    </row>
+    <row r="4659" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4659" s="4"/>
+    </row>
+    <row r="4660" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4660" s="4"/>
+    </row>
+    <row r="4661" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4661" s="4"/>
+    </row>
+    <row r="4662" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4662" s="4"/>
+    </row>
+    <row r="4663" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4663" s="4"/>
+    </row>
+    <row r="4664" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4664" s="4"/>
+    </row>
+    <row r="4665" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4665" s="4"/>
+    </row>
+    <row r="4666" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4666" s="4"/>
+    </row>
+    <row r="4667" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4667" s="4"/>
+    </row>
+    <row r="4668" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4668" s="4"/>
+    </row>
+    <row r="4669" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4669" s="4"/>
+    </row>
+    <row r="4670" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4670" s="4"/>
+    </row>
+    <row r="4671" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4671" s="4"/>
+    </row>
+    <row r="4672" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4672" s="4"/>
+    </row>
+    <row r="4673" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4673" s="4"/>
+    </row>
+    <row r="4674" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4674" s="4"/>
+    </row>
+    <row r="4675" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4675" s="4"/>
+    </row>
+    <row r="4676" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4676" s="4"/>
+    </row>
+    <row r="4677" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4677" s="4"/>
+    </row>
+    <row r="4678" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4678" s="4"/>
+    </row>
+    <row r="4679" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4679" s="4"/>
+    </row>
+    <row r="4680" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4680" s="4"/>
+    </row>
+    <row r="4681" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4681" s="4"/>
+    </row>
+    <row r="4682" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4682" s="4"/>
+    </row>
+    <row r="4683" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4683" s="4"/>
+    </row>
+    <row r="4684" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4684" s="4"/>
+    </row>
+    <row r="4685" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4685" s="4"/>
+    </row>
+    <row r="4686" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4686" s="4"/>
+    </row>
+    <row r="4687" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4687" s="4"/>
+    </row>
+    <row r="4688" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4688" s="4"/>
+    </row>
+    <row r="4689" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4689" s="4"/>
+    </row>
+    <row r="4690" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4690" s="4"/>
+    </row>
+    <row r="4691" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4691" s="4"/>
+    </row>
+    <row r="4692" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4692" s="4"/>
+    </row>
+    <row r="4693" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4693" s="4"/>
+    </row>
+    <row r="4694" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4694" s="4"/>
+    </row>
+    <row r="4695" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4695" s="4"/>
+    </row>
+    <row r="4696" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4696" s="4"/>
+    </row>
+    <row r="4697" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4697" s="4"/>
+    </row>
+    <row r="4698" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4698" s="4"/>
+    </row>
+    <row r="4699" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4699" s="4"/>
+    </row>
+    <row r="4700" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4700" s="4"/>
+    </row>
+    <row r="4701" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4701" s="4"/>
+    </row>
+    <row r="4702" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4702" s="4"/>
+    </row>
+    <row r="4703" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4703" s="4"/>
+    </row>
+    <row r="4704" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4704" s="4"/>
+    </row>
+    <row r="4705" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4705" s="4"/>
+    </row>
+    <row r="4706" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4706" s="4"/>
+    </row>
+    <row r="4707" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4707" s="4"/>
+    </row>
+    <row r="4708" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4708" s="4"/>
+    </row>
+    <row r="4709" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4709" s="4"/>
+    </row>
+    <row r="4710" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4710" s="4"/>
+    </row>
+    <row r="4711" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4711" s="4"/>
+    </row>
+    <row r="4712" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4712" s="4"/>
+    </row>
+    <row r="4713" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4713" s="4"/>
+    </row>
+    <row r="4714" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4714" s="4"/>
+    </row>
+    <row r="4715" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4715" s="4"/>
+    </row>
+    <row r="4716" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4716" s="4"/>
+    </row>
+    <row r="4717" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4717" s="4"/>
+    </row>
+    <row r="4718" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4718" s="4"/>
+    </row>
+    <row r="4719" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4719" s="4"/>
+    </row>
+    <row r="4720" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4720" s="4"/>
+    </row>
+    <row r="4721" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4721" s="4"/>
+    </row>
+    <row r="4722" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4722" s="4"/>
+    </row>
+    <row r="4723" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4723" s="4"/>
+    </row>
+    <row r="4724" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4724" s="4"/>
+    </row>
+    <row r="4725" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4725" s="4"/>
+    </row>
+    <row r="4726" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4726" s="4"/>
+    </row>
+    <row r="4727" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4727" s="4"/>
+    </row>
+    <row r="4728" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4728" s="4"/>
+    </row>
+    <row r="4729" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4729" s="4"/>
+    </row>
+    <row r="4730" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4730" s="4"/>
+    </row>
+    <row r="4731" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4731" s="4"/>
+    </row>
+    <row r="4732" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4732" s="4"/>
+    </row>
+    <row r="4733" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4733" s="4"/>
+    </row>
+    <row r="4734" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4734" s="4"/>
+    </row>
+    <row r="4735" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4735" s="4"/>
+    </row>
+    <row r="4736" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4736" s="4"/>
+    </row>
+    <row r="4737" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4737" s="4"/>
+    </row>
+    <row r="4738" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4738" s="4"/>
+    </row>
+    <row r="4739" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4739" s="4"/>
+    </row>
+    <row r="4740" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4740" s="4"/>
+    </row>
+    <row r="4741" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4741" s="4"/>
+    </row>
+    <row r="4742" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4742" s="4"/>
+    </row>
+    <row r="4743" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4743" s="4"/>
+    </row>
+    <row r="4744" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4744" s="4"/>
+    </row>
+    <row r="4745" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4745" s="4"/>
+    </row>
+    <row r="4746" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4746" s="4"/>
+    </row>
+    <row r="4747" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4747" s="4"/>
+    </row>
+    <row r="4748" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4748" s="4"/>
+    </row>
+    <row r="4749" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4749" s="4"/>
+    </row>
+    <row r="4750" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4750" s="4"/>
+    </row>
+    <row r="4751" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4751" s="4"/>
+    </row>
+    <row r="4752" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4752" s="4"/>
+    </row>
+    <row r="4753" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4753" s="4"/>
+    </row>
+    <row r="4754" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4754" s="4"/>
+    </row>
+    <row r="4755" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4755" s="4"/>
+    </row>
+    <row r="4756" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4756" s="4"/>
+    </row>
+    <row r="4757" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4757" s="4"/>
+    </row>
+    <row r="4758" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4758" s="4"/>
+    </row>
+    <row r="4759" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4759" s="4"/>
+    </row>
+    <row r="4760" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4760" s="4"/>
+    </row>
+    <row r="4761" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4761" s="4"/>
+    </row>
+    <row r="4762" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4762" s="4"/>
+    </row>
+    <row r="4763" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4763" s="4"/>
+    </row>
+    <row r="4764" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4764" s="4"/>
+    </row>
+    <row r="4765" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4765" s="4"/>
+    </row>
+    <row r="4766" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4766" s="4"/>
+    </row>
+    <row r="4767" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4767" s="4"/>
+    </row>
+    <row r="4768" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4768" s="4"/>
+    </row>
+    <row r="4769" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4769" s="4"/>
+    </row>
+    <row r="4770" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4770" s="4"/>
+    </row>
+    <row r="4771" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4771" s="4"/>
+    </row>
+    <row r="4772" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4772" s="4"/>
+    </row>
+    <row r="4773" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4773" s="4"/>
+    </row>
+    <row r="4774" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4774" s="4"/>
+    </row>
+    <row r="4775" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4775" s="4"/>
+    </row>
+    <row r="4776" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4776" s="4"/>
+    </row>
+    <row r="4777" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4777" s="4"/>
+    </row>
+    <row r="4778" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4778" s="4"/>
+    </row>
+    <row r="4779" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4779" s="4"/>
+    </row>
+    <row r="4780" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4780" s="4"/>
+    </row>
+    <row r="4781" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4781" s="4"/>
+    </row>
+    <row r="4782" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4782" s="4"/>
+    </row>
+    <row r="4783" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4783" s="4"/>
+    </row>
+    <row r="4784" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4784" s="4"/>
+    </row>
+    <row r="4785" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4785" s="4"/>
+    </row>
+    <row r="4786" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4786" s="4"/>
+    </row>
+    <row r="4787" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4787" s="4"/>
+    </row>
+    <row r="4788" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4788" s="4"/>
+    </row>
+    <row r="4789" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4789" s="4"/>
+    </row>
+    <row r="4790" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4790" s="4"/>
+    </row>
+    <row r="4791" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4791" s="4"/>
+    </row>
+    <row r="4792" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4792" s="4"/>
+    </row>
+    <row r="4793" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4793" s="4"/>
+    </row>
+    <row r="4794" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4794" s="4"/>
+    </row>
+    <row r="4795" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4795" s="4"/>
+    </row>
+    <row r="4796" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4796" s="4"/>
+    </row>
+    <row r="4797" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4797" s="4"/>
+    </row>
+    <row r="4798" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4798" s="4"/>
+    </row>
+    <row r="4799" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4799" s="4"/>
+    </row>
+    <row r="4800" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4800" s="4"/>
+    </row>
+    <row r="4801" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4801" s="4"/>
+    </row>
+    <row r="4802" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4802" s="4"/>
+    </row>
+    <row r="4803" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4803" s="4"/>
+    </row>
+    <row r="4804" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4804" s="4"/>
+    </row>
+    <row r="4805" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4805" s="4"/>
+    </row>
+    <row r="4806" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4806" s="4"/>
+    </row>
+    <row r="4807" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4807" s="4"/>
+    </row>
+    <row r="4808" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4808" s="4"/>
+    </row>
+    <row r="4809" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4809" s="4"/>
+    </row>
+    <row r="4810" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4810" s="4"/>
+    </row>
+    <row r="4811" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4811" s="4"/>
+    </row>
+    <row r="4812" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4812" s="4"/>
+    </row>
+    <row r="4813" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4813" s="4"/>
+    </row>
+    <row r="4814" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4814" s="4"/>
+    </row>
+    <row r="4815" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4815" s="4"/>
+    </row>
+    <row r="4816" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4816" s="4"/>
+    </row>
+    <row r="4817" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4817" s="4"/>
+    </row>
+    <row r="4818" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4818" s="4"/>
+    </row>
+    <row r="4819" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4819" s="4"/>
+    </row>
+    <row r="4820" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4820" s="4"/>
+    </row>
+    <row r="4821" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4821" s="4"/>
+    </row>
+    <row r="4822" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4822" s="4"/>
+    </row>
+    <row r="4823" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4823" s="4"/>
+    </row>
+    <row r="4824" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4824" s="4"/>
+    </row>
+    <row r="4825" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4825" s="4"/>
+    </row>
+    <row r="4826" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4826" s="4"/>
+    </row>
+    <row r="4827" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4827" s="4"/>
+    </row>
+    <row r="4828" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4828" s="4"/>
+    </row>
+    <row r="4829" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4829" s="4"/>
+    </row>
+    <row r="4830" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4830" s="4"/>
+    </row>
+    <row r="4831" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4831" s="4"/>
+    </row>
+    <row r="4832" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4832" s="4"/>
+    </row>
+    <row r="4833" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4833" s="4"/>
+    </row>
+    <row r="4834" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4834" s="4"/>
+    </row>
+    <row r="4835" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4835" s="4"/>
+    </row>
+    <row r="4836" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4836" s="4"/>
+    </row>
+    <row r="4837" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4837" s="4"/>
+    </row>
+    <row r="4838" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4838" s="4"/>
+    </row>
+    <row r="4839" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4839" s="4"/>
+    </row>
+    <row r="4840" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4840" s="4"/>
+    </row>
+    <row r="4841" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4841" s="4"/>
+    </row>
+    <row r="4842" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4842" s="4"/>
+    </row>
+    <row r="4843" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4843" s="4"/>
+    </row>
+    <row r="4844" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4844" s="4"/>
+    </row>
+    <row r="4845" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4845" s="4"/>
+    </row>
+    <row r="4846" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4846" s="4"/>
+    </row>
+    <row r="4847" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4847" s="4"/>
+    </row>
+    <row r="4848" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4848" s="4"/>
+    </row>
+    <row r="4849" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4849" s="4"/>
+    </row>
+    <row r="4850" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4850" s="4"/>
+    </row>
+    <row r="4851" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4851" s="4"/>
+    </row>
+    <row r="4852" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4852" s="4"/>
+    </row>
+    <row r="4853" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4853" s="4"/>
+    </row>
+    <row r="4854" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4854" s="4"/>
+    </row>
+    <row r="4855" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4855" s="4"/>
+    </row>
+    <row r="4856" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4856" s="4"/>
+    </row>
+    <row r="4857" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4857" s="4"/>
+    </row>
+    <row r="4858" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4858" s="4"/>
+    </row>
+    <row r="4859" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4859" s="4"/>
+    </row>
+    <row r="4860" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4860" s="4"/>
+    </row>
+    <row r="4861" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4861" s="4"/>
+    </row>
+    <row r="4862" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4862" s="4"/>
+    </row>
+    <row r="4863" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4863" s="4"/>
+    </row>
+    <row r="4864" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4864" s="4"/>
+    </row>
+    <row r="4865" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4865" s="4"/>
+    </row>
+    <row r="4866" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4866" s="4"/>
+    </row>
+    <row r="4867" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4867" s="4"/>
+    </row>
+    <row r="4868" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4868" s="4"/>
+    </row>
+    <row r="4869" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4869" s="4"/>
+    </row>
+    <row r="4870" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4870" s="4"/>
+    </row>
+    <row r="4871" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4871" s="4"/>
+    </row>
+    <row r="4872" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4872" s="4"/>
+    </row>
+    <row r="4873" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4873" s="4"/>
+    </row>
+    <row r="4874" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4874" s="4"/>
+    </row>
+    <row r="4875" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4875" s="4"/>
+    </row>
+    <row r="4876" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4876" s="4"/>
+    </row>
+    <row r="4877" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4877" s="4"/>
+    </row>
+    <row r="4878" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4878" s="4"/>
+    </row>
+    <row r="4879" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4879" s="4"/>
+    </row>
+    <row r="4880" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4880" s="4"/>
+    </row>
+    <row r="4881" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4881" s="4"/>
+    </row>
+    <row r="4882" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4882" s="4"/>
+    </row>
+    <row r="4883" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4883" s="4"/>
+    </row>
+    <row r="4884" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4884" s="4"/>
+    </row>
+    <row r="4885" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4885" s="4"/>
+    </row>
+    <row r="4886" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4886" s="4"/>
+    </row>
+    <row r="4887" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4887" s="4"/>
+    </row>
+    <row r="4888" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4888" s="4"/>
+    </row>
+    <row r="4889" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4889" s="4"/>
+    </row>
+    <row r="4890" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4890" s="4"/>
+    </row>
+    <row r="4891" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4891" s="4"/>
+    </row>
+    <row r="4892" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4892" s="4"/>
+    </row>
+    <row r="4893" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4893" s="4"/>
+    </row>
+    <row r="4894" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4894" s="4"/>
+    </row>
+    <row r="4895" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4895" s="4"/>
+    </row>
+    <row r="4896" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4896" s="4"/>
+    </row>
+    <row r="4897" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4897" s="4"/>
+    </row>
+    <row r="4898" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4898" s="4"/>
+    </row>
+    <row r="4899" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4899" s="4"/>
+    </row>
+    <row r="4900" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4900" s="4"/>
+    </row>
+    <row r="4901" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4901" s="4"/>
+    </row>
+    <row r="4902" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4902" s="4"/>
+    </row>
+    <row r="4903" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4903" s="4"/>
+    </row>
+    <row r="4904" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4904" s="4"/>
+    </row>
+    <row r="4905" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4905" s="4"/>
+    </row>
+    <row r="4906" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4906" s="4"/>
+    </row>
+    <row r="4907" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4907" s="4"/>
+    </row>
+    <row r="4908" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4908" s="4"/>
+    </row>
+    <row r="4909" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4909" s="4"/>
+    </row>
+    <row r="4910" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4910" s="4"/>
+    </row>
+    <row r="4911" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4911" s="4"/>
+    </row>
+    <row r="4912" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4912" s="4"/>
+    </row>
+    <row r="4913" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4913" s="4"/>
+    </row>
+    <row r="4914" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4914" s="4"/>
+    </row>
+    <row r="4915" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4915" s="4"/>
+    </row>
+    <row r="4916" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4916" s="4"/>
+    </row>
+    <row r="4917" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4917" s="4"/>
+    </row>
+    <row r="4918" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4918" s="4"/>
+    </row>
+    <row r="4919" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4919" s="4"/>
+    </row>
+    <row r="4920" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4920" s="4"/>
+    </row>
+    <row r="4921" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4921" s="4"/>
+    </row>
+    <row r="4922" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4922" s="4"/>
+    </row>
+    <row r="4923" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4923" s="4"/>
+    </row>
+    <row r="4924" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4924" s="4"/>
+    </row>
+    <row r="4925" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4925" s="4"/>
+    </row>
+    <row r="4926" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4926" s="4"/>
+    </row>
+    <row r="4927" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4927" s="4"/>
+    </row>
+    <row r="4928" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4928" s="4"/>
+    </row>
+    <row r="4929" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4929" s="4"/>
+    </row>
+    <row r="4930" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4930" s="4"/>
+    </row>
+    <row r="4931" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4931" s="4"/>
+    </row>
+    <row r="4932" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4932" s="4"/>
+    </row>
+    <row r="4933" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4933" s="4"/>
+    </row>
+    <row r="4934" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4934" s="4"/>
+    </row>
+    <row r="4935" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4935" s="4"/>
+    </row>
+    <row r="4936" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4936" s="4"/>
+    </row>
+    <row r="4937" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4937" s="4"/>
+    </row>
+    <row r="4938" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4938" s="4"/>
+    </row>
+    <row r="4939" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4939" s="4"/>
+    </row>
+    <row r="4940" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4940" s="4"/>
+    </row>
+    <row r="4941" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4941" s="4"/>
+    </row>
+    <row r="4942" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4942" s="4"/>
+    </row>
+    <row r="4943" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4943" s="4"/>
+    </row>
+    <row r="4944" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4944" s="4"/>
+    </row>
+    <row r="4945" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4945" s="4"/>
+    </row>
+    <row r="4946" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4946" s="4"/>
+    </row>
+    <row r="4947" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4947" s="4"/>
+    </row>
+    <row r="4948" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4948" s="4"/>
+    </row>
+    <row r="4949" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4949" s="4"/>
+    </row>
+    <row r="4950" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4950" s="4"/>
+    </row>
+    <row r="4951" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4951" s="4"/>
+    </row>
+    <row r="4952" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4952" s="4"/>
+    </row>
+    <row r="4953" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4953" s="4"/>
+    </row>
+    <row r="4954" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4954" s="4"/>
+    </row>
+    <row r="4955" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4955" s="4"/>
+    </row>
+    <row r="4956" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4956" s="4"/>
+    </row>
+    <row r="4957" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4957" s="4"/>
+    </row>
+    <row r="4958" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4958" s="4"/>
+    </row>
+    <row r="4959" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4959" s="4"/>
+    </row>
+    <row r="4960" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4960" s="4"/>
+    </row>
+    <row r="4961" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4961" s="4"/>
+    </row>
+    <row r="4962" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4962" s="4"/>
+    </row>
+    <row r="4963" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4963" s="4"/>
+    </row>
+    <row r="4964" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4964" s="4"/>
+    </row>
+    <row r="4965" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4965" s="4"/>
+    </row>
+    <row r="4966" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4966" s="4"/>
+    </row>
+    <row r="4967" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4967" s="4"/>
+    </row>
+    <row r="4968" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4968" s="4"/>
+    </row>
+    <row r="4969" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4969" s="4"/>
+    </row>
+    <row r="4970" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4970" s="4"/>
+    </row>
+    <row r="4971" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4971" s="4"/>
+    </row>
+    <row r="4972" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4972" s="4"/>
+    </row>
+    <row r="4973" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4973" s="4"/>
+    </row>
+    <row r="4974" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4974" s="4"/>
+    </row>
+    <row r="4975" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4975" s="4"/>
+    </row>
+    <row r="4976" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4976" s="4"/>
+    </row>
+    <row r="4977" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4977" s="4"/>
+    </row>
+    <row r="4978" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4978" s="4"/>
+    </row>
+    <row r="4979" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4979" s="4"/>
+    </row>
+    <row r="4980" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4980" s="4"/>
+    </row>
+    <row r="4981" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4981" s="4"/>
+    </row>
+    <row r="4982" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4982" s="4"/>
+    </row>
+    <row r="4983" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4983" s="4"/>
+    </row>
+    <row r="4984" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4984" s="4"/>
+    </row>
+    <row r="4985" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4985" s="4"/>
+    </row>
+    <row r="4986" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4986" s="4"/>
+    </row>
+    <row r="4987" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4987" s="4"/>
+    </row>
+    <row r="4988" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4988" s="4"/>
+    </row>
+    <row r="4989" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4989" s="4"/>
+    </row>
+    <row r="4990" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4990" s="4"/>
+    </row>
+    <row r="4991" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4991" s="4"/>
+    </row>
+    <row r="4992" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4992" s="4"/>
+    </row>
+    <row r="4993" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4993" s="4"/>
+    </row>
+    <row r="4994" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4994" s="4"/>
+    </row>
+    <row r="4995" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4995" s="4"/>
+    </row>
+    <row r="4996" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4996" s="4"/>
+    </row>
+    <row r="4997" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4997" s="4"/>
+    </row>
+    <row r="4998" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4998" s="4"/>
+    </row>
+    <row r="4999" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C4999" s="4"/>
+    </row>
+    <row r="5000" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5000" s="4"/>
+    </row>
+    <row r="5001" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5001" s="4"/>
+    </row>
+    <row r="5002" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5002" s="4"/>
+    </row>
+    <row r="5003" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5003" s="4"/>
+    </row>
+    <row r="5004" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5004" s="4"/>
+    </row>
+    <row r="5005" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5005" s="4"/>
+    </row>
+    <row r="5006" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5006" s="4"/>
+    </row>
+    <row r="5007" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5007" s="4"/>
+    </row>
+    <row r="5008" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5008" s="4"/>
+    </row>
+    <row r="5009" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5009" s="4"/>
+    </row>
+    <row r="5010" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5010" s="4"/>
+    </row>
+    <row r="5011" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5011" s="4"/>
+    </row>
+    <row r="5012" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5012" s="4"/>
+    </row>
+    <row r="5013" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5013" s="4"/>
+    </row>
+    <row r="5014" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5014" s="4"/>
+    </row>
+    <row r="5015" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5015" s="4"/>
+    </row>
+    <row r="5016" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5016" s="4"/>
+    </row>
+    <row r="5017" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5017" s="4"/>
+    </row>
+    <row r="5018" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5018" s="4"/>
+    </row>
+    <row r="5019" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5019" s="4"/>
+    </row>
+    <row r="5020" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5020" s="4"/>
+    </row>
+    <row r="5021" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5021" s="4"/>
+    </row>
+    <row r="5022" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5022" s="4"/>
+    </row>
+    <row r="5023" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5023" s="4"/>
+    </row>
+    <row r="5024" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5024" s="4"/>
+    </row>
+    <row r="5025" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5025" s="4"/>
+    </row>
+    <row r="5026" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5026" s="4"/>
+    </row>
+    <row r="5027" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5027" s="4"/>
+    </row>
+    <row r="5028" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5028" s="4"/>
+    </row>
+    <row r="5029" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5029" s="4"/>
+    </row>
+    <row r="5030" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5030" s="4"/>
+    </row>
+    <row r="5031" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5031" s="4"/>
+    </row>
+    <row r="5032" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5032" s="4"/>
+    </row>
+    <row r="5033" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5033" s="4"/>
+    </row>
+    <row r="5034" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5034" s="4"/>
+    </row>
+    <row r="5035" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5035" s="4"/>
+    </row>
+    <row r="5036" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5036" s="4"/>
+    </row>
+    <row r="5037" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5037" s="4"/>
+    </row>
+    <row r="5038" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5038" s="4"/>
+    </row>
+    <row r="5039" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5039" s="4"/>
+    </row>
+    <row r="5040" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5040" s="4"/>
+    </row>
+    <row r="5041" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5041" s="4"/>
+    </row>
+    <row r="5042" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5042" s="4"/>
+    </row>
+    <row r="5043" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5043" s="4"/>
+    </row>
+    <row r="5044" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5044" s="4"/>
+    </row>
+    <row r="5045" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5045" s="4"/>
+    </row>
+    <row r="5046" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5046" s="4"/>
+    </row>
+    <row r="5047" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5047" s="4"/>
+    </row>
+    <row r="5048" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5048" s="4"/>
+    </row>
+    <row r="5049" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5049" s="4"/>
+    </row>
+    <row r="5050" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5050" s="4"/>
+    </row>
+    <row r="5051" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5051" s="4"/>
+    </row>
+    <row r="5052" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5052" s="4"/>
+    </row>
+    <row r="5053" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5053" s="4"/>
+    </row>
+    <row r="5054" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5054" s="4"/>
+    </row>
+    <row r="5055" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5055" s="4"/>
+    </row>
+    <row r="5056" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5056" s="4"/>
+    </row>
+    <row r="5057" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5057" s="4"/>
+    </row>
+    <row r="5058" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5058" s="4"/>
+    </row>
+    <row r="5059" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5059" s="4"/>
+    </row>
+    <row r="5060" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5060" s="4"/>
+    </row>
+    <row r="5061" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5061" s="4"/>
+    </row>
+    <row r="5062" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5062" s="4"/>
+    </row>
+    <row r="5063" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5063" s="4"/>
+    </row>
+    <row r="5064" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5064" s="4"/>
+    </row>
+    <row r="5065" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5065" s="4"/>
+    </row>
+    <row r="5066" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5066" s="4"/>
+    </row>
+    <row r="5067" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5067" s="4"/>
+    </row>
+    <row r="5068" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5068" s="4"/>
+    </row>
+    <row r="5069" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5069" s="4"/>
+    </row>
+    <row r="5070" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5070" s="4"/>
+    </row>
+    <row r="5071" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5071" s="4"/>
+    </row>
+    <row r="5072" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5072" s="4"/>
+    </row>
+    <row r="5073" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5073" s="4"/>
+    </row>
+    <row r="5074" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5074" s="4"/>
+    </row>
+    <row r="5075" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5075" s="4"/>
+    </row>
+    <row r="5076" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5076" s="4"/>
+    </row>
+    <row r="5077" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5077" s="4"/>
+    </row>
+    <row r="5078" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5078" s="4"/>
+    </row>
+    <row r="5079" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5079" s="4"/>
+    </row>
+    <row r="5080" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5080" s="4"/>
+    </row>
+    <row r="5081" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5081" s="4"/>
+    </row>
+    <row r="5082" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5082" s="4"/>
+    </row>
+    <row r="5083" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5083" s="4"/>
+    </row>
+    <row r="5084" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5084" s="4"/>
+    </row>
+    <row r="5085" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5085" s="4"/>
+    </row>
+    <row r="5086" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5086" s="4"/>
+    </row>
+    <row r="5087" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5087" s="4"/>
+    </row>
+    <row r="5088" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5088" s="4"/>
+    </row>
+    <row r="5089" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5089" s="4"/>
+    </row>
+    <row r="5090" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5090" s="4"/>
+    </row>
+    <row r="5091" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5091" s="4"/>
+    </row>
+    <row r="5092" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5092" s="4"/>
+    </row>
+    <row r="5093" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5093" s="4"/>
+    </row>
+    <row r="5094" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5094" s="4"/>
+    </row>
+    <row r="5095" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5095" s="4"/>
+    </row>
+    <row r="5096" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5096" s="4"/>
+    </row>
+    <row r="5097" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5097" s="4"/>
+    </row>
+    <row r="5098" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5098" s="4"/>
+    </row>
+    <row r="5099" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5099" s="4"/>
+    </row>
+    <row r="5100" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5100" s="4"/>
+    </row>
+    <row r="5101" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5101" s="4"/>
+    </row>
+    <row r="5102" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5102" s="4"/>
+    </row>
+    <row r="5103" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5103" s="4"/>
+    </row>
+    <row r="5104" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5104" s="4"/>
+    </row>
+    <row r="5105" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5105" s="4"/>
+    </row>
+    <row r="5106" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5106" s="4"/>
+    </row>
+    <row r="5107" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5107" s="4"/>
+    </row>
+    <row r="5108" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5108" s="4"/>
+    </row>
+    <row r="5109" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5109" s="4"/>
+    </row>
+    <row r="5110" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5110" s="4"/>
+    </row>
+    <row r="5111" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5111" s="4"/>
+    </row>
+    <row r="5112" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5112" s="4"/>
+    </row>
+    <row r="5113" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5113" s="4"/>
+    </row>
+    <row r="5114" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5114" s="4"/>
+    </row>
+    <row r="5115" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5115" s="4"/>
+    </row>
+    <row r="5116" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5116" s="4"/>
+    </row>
+    <row r="5117" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5117" s="4"/>
+    </row>
+    <row r="5118" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5118" s="4"/>
+    </row>
+    <row r="5119" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5119" s="4"/>
+    </row>
+    <row r="5120" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5120" s="4"/>
+    </row>
+    <row r="5121" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5121" s="4"/>
+    </row>
+    <row r="5122" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5122" s="4"/>
+    </row>
+    <row r="5123" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5123" s="4"/>
+    </row>
+    <row r="5124" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5124" s="4"/>
+    </row>
+    <row r="5125" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5125" s="4"/>
+    </row>
+    <row r="5126" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5126" s="4"/>
+    </row>
+    <row r="5127" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5127" s="4"/>
+    </row>
+    <row r="5128" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5128" s="4"/>
+    </row>
+    <row r="5129" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5129" s="4"/>
+    </row>
+    <row r="5130" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5130" s="4"/>
+    </row>
+    <row r="5131" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5131" s="4"/>
+    </row>
+    <row r="5132" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5132" s="4"/>
+    </row>
+    <row r="5133" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5133" s="4"/>
+    </row>
+    <row r="5134" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5134" s="4"/>
+    </row>
+    <row r="5135" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5135" s="4"/>
+    </row>
+    <row r="5136" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5136" s="4"/>
+    </row>
+    <row r="5137" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5137" s="4"/>
+    </row>
+    <row r="5138" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5138" s="4"/>
+    </row>
+    <row r="5139" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5139" s="4"/>
+    </row>
+    <row r="5140" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5140" s="4"/>
+    </row>
+    <row r="5141" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5141" s="4"/>
+    </row>
+    <row r="5142" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5142" s="4"/>
+    </row>
+    <row r="5143" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5143" s="4"/>
+    </row>
+    <row r="5144" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5144" s="4"/>
+    </row>
+    <row r="5145" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5145" s="4"/>
+    </row>
+    <row r="5146" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5146" s="4"/>
+    </row>
+    <row r="5147" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5147" s="4"/>
+    </row>
+    <row r="5148" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5148" s="4"/>
+    </row>
+    <row r="5149" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5149" s="4"/>
+    </row>
+    <row r="5150" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5150" s="4"/>
+    </row>
+    <row r="5151" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5151" s="4"/>
+    </row>
+    <row r="5152" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5152" s="4"/>
+    </row>
+    <row r="5153" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5153" s="4"/>
+    </row>
+    <row r="5154" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5154" s="4"/>
+    </row>
+    <row r="5155" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5155" s="4"/>
+    </row>
+    <row r="5156" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5156" s="4"/>
+    </row>
+    <row r="5157" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5157" s="4"/>
+    </row>
+    <row r="5158" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5158" s="4"/>
+    </row>
+    <row r="5159" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5159" s="4"/>
+    </row>
+    <row r="5160" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5160" s="4"/>
+    </row>
+    <row r="5161" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5161" s="4"/>
+    </row>
+    <row r="5162" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5162" s="4"/>
+    </row>
+    <row r="5163" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5163" s="4"/>
+    </row>
+    <row r="5164" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5164" s="4"/>
+    </row>
+    <row r="5165" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5165" s="4"/>
+    </row>
+    <row r="5166" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5166" s="4"/>
+    </row>
+    <row r="5167" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5167" s="4"/>
+    </row>
+    <row r="5168" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5168" s="4"/>
+    </row>
+    <row r="5169" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5169" s="4"/>
+    </row>
+    <row r="5170" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5170" s="4"/>
+    </row>
+    <row r="5171" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5171" s="4"/>
+    </row>
+    <row r="5172" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5172" s="4"/>
+    </row>
+    <row r="5173" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5173" s="4"/>
+    </row>
+    <row r="5174" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5174" s="4"/>
+    </row>
+    <row r="5175" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5175" s="4"/>
+    </row>
+    <row r="5176" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5176" s="4"/>
+    </row>
+    <row r="5177" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5177" s="4"/>
+    </row>
+    <row r="5178" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5178" s="4"/>
+    </row>
+    <row r="5179" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5179" s="4"/>
+    </row>
+    <row r="5180" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5180" s="4"/>
+    </row>
+    <row r="5181" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5181" s="4"/>
+    </row>
+    <row r="5182" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5182" s="4"/>
+    </row>
+    <row r="5183" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5183" s="4"/>
+    </row>
+    <row r="5184" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5184" s="4"/>
+    </row>
+    <row r="5185" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5185" s="4"/>
+    </row>
+    <row r="5186" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5186" s="4"/>
+    </row>
+    <row r="5187" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5187" s="4"/>
+    </row>
+    <row r="5188" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5188" s="4"/>
+    </row>
+    <row r="5189" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5189" s="4"/>
+    </row>
+    <row r="5190" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5190" s="4"/>
+    </row>
+    <row r="5191" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5191" s="4"/>
+    </row>
+    <row r="5192" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5192" s="4"/>
+    </row>
+    <row r="5193" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5193" s="4"/>
+    </row>
+    <row r="5194" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5194" s="4"/>
+    </row>
+    <row r="5195" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5195" s="4"/>
+    </row>
+    <row r="5196" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5196" s="4"/>
+    </row>
+    <row r="5197" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5197" s="4"/>
+    </row>
+    <row r="5198" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5198" s="4"/>
+    </row>
+    <row r="5199" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5199" s="4"/>
+    </row>
+    <row r="5200" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5200" s="4"/>
+    </row>
+    <row r="5201" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5201" s="4"/>
+    </row>
+    <row r="5202" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5202" s="4"/>
+    </row>
+    <row r="5203" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5203" s="4"/>
+    </row>
+    <row r="5204" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5204" s="4"/>
+    </row>
+    <row r="5205" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5205" s="4"/>
+    </row>
+    <row r="5206" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5206" s="4"/>
+    </row>
+    <row r="5207" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5207" s="4"/>
+    </row>
+    <row r="5208" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5208" s="4"/>
+    </row>
+    <row r="5209" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5209" s="4"/>
+    </row>
+    <row r="5210" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5210" s="4"/>
+    </row>
+    <row r="5211" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5211" s="4"/>
+    </row>
+    <row r="5212" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5212" s="4"/>
+    </row>
+    <row r="5213" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5213" s="4"/>
+    </row>
+    <row r="5214" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5214" s="4"/>
+    </row>
+    <row r="5215" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5215" s="4"/>
+    </row>
+    <row r="5216" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5216" s="4"/>
+    </row>
+    <row r="5217" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5217" s="4"/>
+    </row>
+    <row r="5218" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5218" s="4"/>
+    </row>
+    <row r="5219" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5219" s="4"/>
+    </row>
+    <row r="5220" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5220" s="4"/>
+    </row>
+    <row r="5221" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5221" s="4"/>
+    </row>
+    <row r="5222" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5222" s="4"/>
+    </row>
+    <row r="5223" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5223" s="4"/>
+    </row>
+    <row r="5224" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5224" s="4"/>
+    </row>
+    <row r="5225" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5225" s="4"/>
+    </row>
+    <row r="5226" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C5226" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <customProperties>

</xml_diff>